<commit_message>
Slice 3.5 — assets from handover protocols, and the date that was a placeholder
A confirmed protocol writes the real handover date; the register never carried one.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/model/dona-building-unit-model-draft.xlsx
+++ b/docs/model/dona-building-unit-model-draft.xlsx
@@ -4561,12 +4561,12 @@
       <c r="E88" s="6" t="inlineStr"/>
       <c r="F88" s="6" t="inlineStr">
         <is>
-          <t>The specific kind, from a controlled list.</t>
+          <t>FIXTURE: AC · WATER_HEATER · OVEN · BLINDS · PLUMBING. SAFETY: EXTINGUISHER · SPRINKLER · SMOKE_DETECTOR · EMERGENCY_LIGHT · MAMAD_BLAST_DOOR. UTILITY: PUMP · ELEVATOR · BOILER · GATE_MOTOR · INTERCOM · METER.</t>
         </is>
       </c>
       <c r="G88" s="6" t="inlineStr">
         <is>
-          <t>This is the field the responsibility matrix keys on. It must be a list, never free text — and unlike obligation types, this list is governed, not admin-editable. Editing it edits policy.</t>
+          <t>This is the field the responsibility matrix keys on. It must be a list, never free text — and unlike obligation types, this list is governed, not admin-editable. Editing it edits policy. The pairs are the workbook's own class examples, enumerated rather than left as prose, because a governed list that is nowhere written down is not governed. A composite CHECK on the pair stops a SAFETY sprinkler being filed as a FIXTURE.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Slice 3.5 — assets from handover protocols, and the date that was a placeholder (#46)
A confirmed protocol writes the real handover date; the register never carried one.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/model/dona-building-unit-model-draft.xlsx
+++ b/docs/model/dona-building-unit-model-draft.xlsx
@@ -4561,12 +4561,12 @@
       <c r="E88" s="6" t="inlineStr"/>
       <c r="F88" s="6" t="inlineStr">
         <is>
-          <t>The specific kind, from a controlled list.</t>
+          <t>FIXTURE: AC · WATER_HEATER · OVEN · BLINDS · PLUMBING. SAFETY: EXTINGUISHER · SPRINKLER · SMOKE_DETECTOR · EMERGENCY_LIGHT · MAMAD_BLAST_DOOR. UTILITY: PUMP · ELEVATOR · BOILER · GATE_MOTOR · INTERCOM · METER.</t>
         </is>
       </c>
       <c r="G88" s="6" t="inlineStr">
         <is>
-          <t>This is the field the responsibility matrix keys on. It must be a list, never free text — and unlike obligation types, this list is governed, not admin-editable. Editing it edits policy.</t>
+          <t>This is the field the responsibility matrix keys on. It must be a list, never free text — and unlike obligation types, this list is governed, not admin-editable. Editing it edits policy. The pairs are the workbook's own class examples, enumerated rather than left as prose, because a governed list that is nowhere written down is not governed. A composite CHECK on the pair stops a SAFETY sprinkler being filed as a FIXTURE.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Slice 3.6 — find a named lease in four seconds
Search is extended, not forked. The guard verdict lives on the document row so
the panel does not scrape audit_log or re-read the bucket.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/model/dona-building-unit-model-draft.xlsx
+++ b/docs/model/dona-building-unit-model-draft.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ENTITIES'!$A$1:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RELATIONSHIPS'!$A$1:$H$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'FIELDS'!$A$1:$G$135</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'FIELDS'!$A$1:$G$136</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ADMIN VIEWS'!$A$1:$E$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DECISIONS'!$A$1:$E$8</definedName>
   </definedNames>
@@ -2010,7 +2010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G135"/>
+  <dimension ref="A1:G136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5137,47 +5137,51 @@
       <c r="F107" s="6" t="inlineStr"/>
       <c r="G107" s="6" t="inlineStr"/>
     </row>
-    <row r="108" ht="20" customHeight="1">
-      <c r="A108" s="7" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>verification_verdict</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E108" s="6" t="inlineStr"/>
+      <c r="F108" s="6" t="inlineStr">
+        <is>
+          <t>verified · unverified · unguarded</t>
+        </is>
+      </c>
+      <c r="G108" s="6" t="inlineStr">
+        <is>
+          <t>Slice 3.6. The 3.3 guard's result, made a property of a list so a scan does not look identical to a lease whose marker terms were found. Not figure 5's state (RECEIVED / EXTRACTED / ACCEPTED / REJECTED), which is still omitted: refused uploads still leave no row. 4.1 may later move unverified → verified once OCR gives the file a text layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="20" customHeight="1">
+      <c r="A109" s="7" t="inlineStr">
         <is>
           <t>E13 · DOCUMENTLINK — one document, several bindings</t>
         </is>
       </c>
-      <c r="B108" s="8" t="n"/>
-      <c r="C108" s="8" t="n"/>
-      <c r="D108" s="8" t="n"/>
-      <c r="E108" s="8" t="n"/>
-      <c r="F108" s="8" t="n"/>
-      <c r="G108" s="8" t="n"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="6" t="inlineStr">
-        <is>
-          <t>DocumentLink</t>
-        </is>
-      </c>
-      <c r="B109" s="6" t="inlineStr">
-        <is>
-          <t>document_id</t>
-        </is>
-      </c>
-      <c r="C109" s="6" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D109" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E109" s="6" t="inlineStr">
-        <is>
-          <t>PK part, FK</t>
-        </is>
-      </c>
-      <c r="F109" s="6" t="inlineStr"/>
-      <c r="G109" s="6" t="inlineStr"/>
+      <c r="B109" s="8" t="n"/>
+      <c r="C109" s="8" t="n"/>
+      <c r="D109" s="8" t="n"/>
+      <c r="E109" s="8" t="n"/>
+      <c r="F109" s="8" t="n"/>
+      <c r="G109" s="8" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
@@ -5187,12 +5191,12 @@
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>entity_type</t>
+          <t>document_id</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D110" s="6" t="inlineStr">
@@ -5200,17 +5204,13 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E110" s="6" t="inlineStr"/>
-      <c r="F110" s="6" t="inlineStr">
-        <is>
-          <t>PROJECT · BUILDING · SPACE · UNIT · TENANCY · PARTY · ASSET · OBLIGATION</t>
-        </is>
-      </c>
-      <c r="G110" s="6" t="inlineStr">
-        <is>
-          <t>PROJECT added by D2 — a tender document belongs to the project, not to any one building.</t>
-        </is>
-      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>PK part, FK</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="inlineStr"/>
+      <c r="G110" s="6" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
@@ -5220,12 +5220,12 @@
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>entity_id</t>
+          <t>entity_type</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
@@ -5233,13 +5233,17 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E111" s="6" t="inlineStr">
-        <is>
-          <t>PK part</t>
-        </is>
-      </c>
-      <c r="F111" s="6" t="inlineStr"/>
-      <c r="G111" s="6" t="inlineStr"/>
+      <c r="E111" s="6" t="inlineStr"/>
+      <c r="F111" s="6" t="inlineStr">
+        <is>
+          <t>PROJECT · BUILDING · SPACE · UNIT · TENANCY · PARTY · ASSET · OBLIGATION</t>
+        </is>
+      </c>
+      <c r="G111" s="6" t="inlineStr">
+        <is>
+          <t>PROJECT added by D2 — a tender document belongs to the project, not to any one building.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
@@ -5249,72 +5253,72 @@
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
+          <t>entity_id</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E112" s="6" t="inlineStr">
+        <is>
+          <t>PK part</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="inlineStr"/>
+      <c r="G112" s="6" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>DocumentLink</t>
+        </is>
+      </c>
+      <c r="B113" s="6" t="inlineStr">
+        <is>
           <t>link_role</t>
         </is>
       </c>
-      <c r="C112" s="6" t="inlineStr">
+      <c r="C113" s="6" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
       </c>
-      <c r="D112" s="6" t="inlineStr">
+      <c r="D113" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="E112" s="6" t="inlineStr"/>
-      <c r="F112" s="6" t="inlineStr">
+      <c r="E113" s="6" t="inlineStr"/>
+      <c r="F113" s="6" t="inlineStr">
         <is>
           <t>SIGNATORY · SUBJECT · EVIDENCE · SOURCE</t>
         </is>
       </c>
-      <c r="G112" s="6" t="inlineStr">
+      <c r="G113" s="6" t="inlineStr">
         <is>
           <t>A lease links to two parties as SIGNATORY and to the unit as SUBJECT.</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="7" t="inlineStr">
+    <row r="114" ht="20" customHeight="1">
+      <c r="A114" s="7" t="inlineStr">
         <is>
           <t>E14 · PROVIDER — stub only, out of scope this pass</t>
         </is>
       </c>
-      <c r="B113" s="8" t="n"/>
-      <c r="C113" s="8" t="n"/>
-      <c r="D113" s="8" t="n"/>
-      <c r="E113" s="8" t="n"/>
-      <c r="F113" s="8" t="n"/>
-      <c r="G113" s="8" t="n"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="6" t="inlineStr">
-        <is>
-          <t>Provider</t>
-        </is>
-      </c>
-      <c r="B114" s="6" t="inlineStr">
-        <is>
-          <t>provider_id</t>
-        </is>
-      </c>
-      <c r="C114" s="6" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D114" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E114" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F114" s="6" t="inlineStr"/>
-      <c r="G114" s="6" t="inlineStr"/>
+      <c r="B114" s="8" t="n"/>
+      <c r="C114" s="8" t="n"/>
+      <c r="D114" s="8" t="n"/>
+      <c r="E114" s="8" t="n"/>
+      <c r="F114" s="8" t="n"/>
+      <c r="G114" s="8" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
@@ -5324,12 +5328,12 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>provider_id</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
@@ -5337,7 +5341,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E115" s="6" t="inlineStr"/>
+      <c r="E115" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="F115" s="6" t="inlineStr"/>
       <c r="G115" s="6" t="inlineStr"/>
     </row>
@@ -5349,72 +5357,68 @@
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D116" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E116" s="6" t="inlineStr"/>
+      <c r="F116" s="6" t="inlineStr"/>
+      <c r="G116" s="6" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="B117" s="6" t="inlineStr">
+        <is>
           <t>provider_kind</t>
         </is>
       </c>
-      <c r="C116" s="6" t="inlineStr">
+      <c r="C117" s="6" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
       </c>
-      <c r="D116" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E116" s="6" t="inlineStr"/>
-      <c r="F116" s="6" t="inlineStr">
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E117" s="6" t="inlineStr"/>
+      <c r="F117" s="6" t="inlineStr">
         <is>
           <t>IN_HOUSE_CREW · CONTRACTOR · DEVELOPER_WARRANTY</t>
         </is>
       </c>
-      <c r="G116" s="6" t="inlineStr">
+      <c r="G117" s="6" t="inlineStr">
         <is>
           <t>Present only to make R11 resolvable. Everything else about providers waits.</t>
         </is>
       </c>
     </row>
-    <row r="117" ht="20" customHeight="1">
-      <c r="A117" s="7" t="inlineStr">
+    <row r="118" ht="20" customHeight="1">
+      <c r="A118" s="7" t="inlineStr">
         <is>
           <t>E15 · DOCUMENTTYPE — the catalogue behind Document (A8)</t>
         </is>
       </c>
-      <c r="B117" s="8" t="n"/>
-      <c r="C117" s="8" t="n"/>
-      <c r="D117" s="8" t="n"/>
-      <c r="E117" s="8" t="n"/>
-      <c r="F117" s="8" t="n"/>
-      <c r="G117" s="8" t="n"/>
-    </row>
-    <row r="118">
-      <c r="A118" s="6" t="inlineStr">
-        <is>
-          <t>DocumentType</t>
-        </is>
-      </c>
-      <c r="B118" s="6" t="inlineStr">
-        <is>
-          <t>document_type_id</t>
-        </is>
-      </c>
-      <c r="C118" s="6" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D118" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E118" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F118" s="6" t="inlineStr"/>
-      <c r="G118" s="6" t="inlineStr"/>
+      <c r="B118" s="8" t="n"/>
+      <c r="C118" s="8" t="n"/>
+      <c r="D118" s="8" t="n"/>
+      <c r="E118" s="8" t="n"/>
+      <c r="F118" s="8" t="n"/>
+      <c r="G118" s="8" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
@@ -5424,12 +5428,12 @@
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>type_key</t>
+          <t>document_type_id</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
@@ -5439,19 +5443,11 @@
       </c>
       <c r="E119" s="6" t="inlineStr">
         <is>
-          <t>unique</t>
-        </is>
-      </c>
-      <c r="F119" s="6" t="inlineStr">
-        <is>
-          <t>Stable machine key. Nine seed rows: lease · lease_amendment · termination_notice · arnona · insurance · id · bank_guarantee · handover_protocol · inspection_certificate.</t>
-        </is>
-      </c>
-      <c r="G119" s="6" t="inlineStr">
-        <is>
-          <t>The first eight are the Data Model's. inspection_certificate is the ninth, needed by SAFETY assets and by the compliance tab. Never renamed and never reused — filed documents point at it.</t>
-        </is>
-      </c>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="inlineStr"/>
+      <c r="G119" s="6" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
@@ -5461,7 +5457,7 @@
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>label_he</t>
+          <t>type_key</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
@@ -5474,13 +5470,21 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E120" s="6" t="inlineStr"/>
+      <c r="E120" s="6" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
       <c r="F120" s="6" t="inlineStr">
         <is>
-          <t>What the admin sees and chooses from: חוזה שכירות · נספח · הודעת סיום · ארנונה · ביטוח · תעודת זהות · ערבות בנקאית · פרוטוקול מסירה · תעודת בדיקה.</t>
-        </is>
-      </c>
-      <c r="G120" s="6" t="inlineStr"/>
+          <t>Stable machine key. Nine seed rows: lease · lease_amendment · termination_notice · arnona · insurance · id · bank_guarantee · handover_protocol · inspection_certificate.</t>
+        </is>
+      </c>
+      <c r="G120" s="6" t="inlineStr">
+        <is>
+          <t>The first eight are the Data Model's. inspection_certificate is the ninth, needed by SAFETY assets and by the compliance tab. Never renamed and never reused — filed documents point at it.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
@@ -5490,7 +5494,7 @@
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>label_en</t>
+          <t>label_he</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
@@ -5500,11 +5504,15 @@
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E121" s="6" t="inlineStr"/>
-      <c r="F121" s="6" t="inlineStr"/>
+      <c r="F121" s="6" t="inlineStr">
+        <is>
+          <t>What the admin sees and chooses from: חוזה שכירות · נספח · הודעת סיום · ארנונה · ביטוח · תעודת זהות · ערבות בנקאית · פרוטוקול מסירה · תעודת בדיקה.</t>
+        </is>
+      </c>
       <c r="G121" s="6" t="inlineStr"/>
     </row>
     <row r="122">
@@ -5515,12 +5523,12 @@
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>verification_terms</t>
+          <t>label_en</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
         <is>
-          <t>text[]</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D122" s="6" t="inlineStr">
@@ -5529,16 +5537,8 @@
         </is>
       </c>
       <c r="E122" s="6" t="inlineStr"/>
-      <c r="F122" s="6" t="inlineStr">
-        <is>
-          <t>Marker terms a document of this type is expected to contain.</t>
-        </is>
-      </c>
-      <c r="G122" s="6" t="inlineStr">
-        <is>
-          <t>The cheap guard in slice 3.3 — right slot, wrong file — reads this and nothing else. It lives on the type row rather than in code, or a new type would arrive with no guard until the next release, and A8 would be true of the catalogue and false of everything that uses it.</t>
-        </is>
-      </c>
+      <c r="F122" s="6" t="inlineStr"/>
+      <c r="G122" s="6" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
@@ -5548,28 +5548,28 @@
       </c>
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>verification_terms</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>text[]</t>
         </is>
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E123" s="6" t="inlineStr"/>
       <c r="F123" s="6" t="inlineStr">
         <is>
-          <t>Retired types stay as rows and stop appearing in the 'file a document' list.</t>
+          <t>Marker terms a document of this type is expected to contain.</t>
         </is>
       </c>
       <c r="G123" s="6" t="inlineStr">
         <is>
-          <t>NEVER delete a type. A9: the admin screen for this catalogue lands in month two; until then we add rows through seeds, which is the same mechanism with a different hand on it.</t>
+          <t>The cheap guard in slice 3.3 — right slot, wrong file — reads this and nothing else. It lives on the type row rather than in code, or a new type would arrive with no guard until the next release, and A8 would be true of the catalogue and false of everything that uses it.</t>
         </is>
       </c>
     </row>
@@ -5581,72 +5581,76 @@
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>is_active</t>
         </is>
       </c>
       <c r="C124" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D124" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E124" s="6" t="inlineStr"/>
       <c r="F124" s="6" t="inlineStr">
         <is>
+          <t>Retired types stay as rows and stop appearing in the 'file a document' list.</t>
+        </is>
+      </c>
+      <c r="G124" s="6" t="inlineStr">
+        <is>
+          <t>NEVER delete a type. A9: the admin screen for this catalogue lands in month two; until then we add rows through seeds, which is the same mechanism with a different hand on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>DocumentType</t>
+        </is>
+      </c>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D125" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E125" s="6" t="inlineStr"/>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
           <t>NO promotes_to. NO validation_rules. NO renewal_cadence.</t>
         </is>
       </c>
-      <c r="G124" s="6" t="inlineStr">
+      <c r="G125" s="6" t="inlineStr">
         <is>
           <t>A8 deliberately: a promotes_to column would make promotion a row, and promotion is the half that is governed — it costs a migration and a reviewed mapping because those columns are what the isolation join, the responsibility matrix and the state machine read. Renewal cadence and 'what is missing' belong to DocumentRequirement, which is month two's.</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="20" customHeight="1">
-      <c r="A125" s="7" t="inlineStr">
+    <row r="126" ht="20" customHeight="1">
+      <c r="A126" s="7" t="inlineStr">
         <is>
           <t>E16 · DOCUMENTTYPEFIELD — what a type declares, in one version (A8)</t>
         </is>
       </c>
-      <c r="B125" s="8" t="n"/>
-      <c r="C125" s="8" t="n"/>
-      <c r="D125" s="8" t="n"/>
-      <c r="E125" s="8" t="n"/>
-      <c r="F125" s="8" t="n"/>
-      <c r="G125" s="8" t="n"/>
-    </row>
-    <row r="126">
-      <c r="A126" s="6" t="inlineStr">
-        <is>
-          <t>DocumentTypeField</t>
-        </is>
-      </c>
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>document_type_field_id</t>
-        </is>
-      </c>
-      <c r="C126" s="6" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D126" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E126" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F126" s="6" t="inlineStr"/>
-      <c r="G126" s="6" t="inlineStr"/>
+      <c r="B126" s="8" t="n"/>
+      <c r="C126" s="8" t="n"/>
+      <c r="D126" s="8" t="n"/>
+      <c r="E126" s="8" t="n"/>
+      <c r="F126" s="8" t="n"/>
+      <c r="G126" s="8" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
@@ -5656,7 +5660,7 @@
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>document_type_id</t>
+          <t>document_type_field_id</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
@@ -5671,15 +5675,11 @@
       </c>
       <c r="E127" s="6" t="inlineStr">
         <is>
-          <t>FK → DocumentType</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="F127" s="6" t="inlineStr"/>
-      <c r="G127" s="6" t="inlineStr">
-        <is>
-          <t>See R18.</t>
-        </is>
-      </c>
+      <c r="G127" s="6" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
@@ -5689,12 +5689,12 @@
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>field_key</t>
+          <t>document_type_id</t>
         </is>
       </c>
       <c r="C128" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D128" s="6" t="inlineStr">
@@ -5704,17 +5704,13 @@
       </c>
       <c r="E128" s="6" t="inlineStr">
         <is>
-          <t>unique part</t>
-        </is>
-      </c>
-      <c r="F128" s="6" t="inlineStr">
-        <is>
-          <t>Stable machine key within the type: start_date, end_date, tenant_name, apartment_number.</t>
-        </is>
-      </c>
+          <t>FK → DocumentType</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr"/>
       <c r="G128" s="6" t="inlineStr">
         <is>
-          <t>Unique on (document_type_id, field_key, effective_from) — the same field, redeclared, is a new row and not an edit.</t>
+          <t>See R18.</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5722,7 @@
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>label_he</t>
+          <t>field_key</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
@@ -5739,13 +5735,21 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E129" s="6" t="inlineStr"/>
+      <c r="E129" s="6" t="inlineStr">
+        <is>
+          <t>unique part</t>
+        </is>
+      </c>
       <c r="F129" s="6" t="inlineStr">
         <is>
-          <t>What a reviewer sees beside the value on the page.</t>
-        </is>
-      </c>
-      <c r="G129" s="6" t="inlineStr"/>
+          <t>Stable machine key within the type: start_date, end_date, tenant_name, apartment_number.</t>
+        </is>
+      </c>
+      <c r="G129" s="6" t="inlineStr">
+        <is>
+          <t>Unique on (document_type_id, field_key, effective_from) — the same field, redeclared, is a new row and not an edit.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
@@ -5755,12 +5759,12 @@
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>value_type</t>
+          <t>label_he</t>
         </is>
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D130" s="6" t="inlineStr">
@@ -5771,14 +5775,10 @@
       <c r="E130" s="6" t="inlineStr"/>
       <c r="F130" s="6" t="inlineStr">
         <is>
-          <t>TEXT · NUMBER · DATE · BOOLEAN · ENUM</t>
-        </is>
-      </c>
-      <c r="G130" s="6" t="inlineStr">
-        <is>
-          <t>No MONEY type, and no money field is seeded. READ ME rule 3 binds hardest at promotion: no amount is ever a column on a business record, and no amount is ever quoted to a tenant — the golden set carries that as a standing refusal case.</t>
-        </is>
-      </c>
+          <t>What a reviewer sees beside the value on the page.</t>
+        </is>
+      </c>
+      <c r="G130" s="6" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
@@ -5788,12 +5788,12 @@
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
-          <t>is_required</t>
+          <t>value_type</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="D131" s="6" t="inlineStr">
@@ -5804,12 +5804,12 @@
       <c r="E131" s="6" t="inlineStr"/>
       <c r="F131" s="6" t="inlineStr">
         <is>
-          <t>Is this field expected in a document of this type?</t>
+          <t>TEXT · NUMBER · DATE · BOOLEAN · ENUM</t>
         </is>
       </c>
       <c r="G131" s="6" t="inlineStr">
         <is>
-          <t>A missing required field is a RESULT, not an error. A lease commonly names no guarantor — SPEC-flows A2 — and extraction returning nothing there is correct.</t>
+          <t>No MONEY type, and no money field is seeded. READ ME rule 3 binds hardest at promotion: no amount is ever a column on a business record, and no amount is ever quoted to a tenant — the golden set carries that as a standing refusal case.</t>
         </is>
       </c>
     </row>
@@ -5821,28 +5821,28 @@
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>extraction_hint</t>
+          <t>is_required</t>
         </is>
       </c>
       <c r="C132" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D132" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E132" s="6" t="inlineStr"/>
       <c r="F132" s="6" t="inlineStr">
         <is>
-          <t>The Hebrew phrasing as printed on the form, to look for on the page.</t>
+          <t>Is this field expected in a document of this type?</t>
         </is>
       </c>
       <c r="G132" s="6" t="inlineStr">
         <is>
-          <t>A hint, never a key. Same rule as a Drive path.</t>
+          <t>A missing required field is a RESULT, not an error. A lease commonly names no guarantor — SPEC-flows A2 — and extraction returning nothing there is correct.</t>
         </is>
       </c>
     </row>
@@ -5854,28 +5854,28 @@
       </c>
       <c r="B133" s="6" t="inlineStr">
         <is>
-          <t>effective_from</t>
+          <t>extraction_hint</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E133" s="6" t="inlineStr"/>
       <c r="F133" s="6" t="inlineStr">
         <is>
-          <t>The version. This row governs values extracted on or after this date.</t>
+          <t>The Hebrew phrasing as printed on the form, to look for on the page.</t>
         </is>
       </c>
       <c r="G133" s="6" t="inlineStr">
         <is>
-          <t>A8, for policy_version_id's reason. The extracted value points at THIS row, so A8's schema_version_id is document_type_field_id and there is no separate version entity.</t>
+          <t>A hint, never a key. Same rule as a Drive path.</t>
         </is>
       </c>
     </row>
@@ -5887,7 +5887,7 @@
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>effective_to</t>
+          <t>effective_from</t>
         </is>
       </c>
       <c r="C134" s="6" t="inlineStr">
@@ -5897,18 +5897,18 @@
       </c>
       <c r="D134" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E134" s="6" t="inlineStr"/>
       <c r="F134" s="6" t="inlineStr">
         <is>
-          <t>Null = the current declaration.</t>
+          <t>The version. This row governs values extracted on or after this date.</t>
         </is>
       </c>
       <c r="G134" s="6" t="inlineStr">
         <is>
-          <t>Closing a row never edits it. Nothing is overwritten — READ ME rule 2.</t>
+          <t>A8, for policy_version_id's reason. The extracted value points at THIS row, so A8's schema_version_id is document_type_field_id and there is no separate version entity.</t>
         </is>
       </c>
     </row>
@@ -5920,33 +5920,66 @@
       </c>
       <c r="B135" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>effective_to</t>
         </is>
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E135" s="6" t="inlineStr"/>
       <c r="F135" s="6" t="inlineStr">
         <is>
+          <t>Null = the current declaration.</t>
+        </is>
+      </c>
+      <c r="G135" s="6" t="inlineStr">
+        <is>
+          <t>Closing a row never edits it. Nothing is overwritten — READ ME rule 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="6" t="inlineStr">
+        <is>
+          <t>DocumentTypeField</t>
+        </is>
+      </c>
+      <c r="B136" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C136" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D136" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E136" s="6" t="inlineStr"/>
+      <c r="F136" s="6" t="inlineStr">
+        <is>
           <t>NO target column, NO promotion mapping.</t>
         </is>
       </c>
-      <c r="G135" s="6" t="inlineStr">
+      <c r="G136" s="6" t="inlineStr">
         <is>
           <t>Capture is open; promotion is governed. The mapping from a captured field to a typed column is a migration and a reviewed mapping, not a row an admin can add on a Tuesday. See A8.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G135"/>
+  <autoFilter ref="A1:G136"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Slice 3.6 — find a named lease in four seconds (#47)
Search is extended, not forked. The guard verdict lives on the document row so
the panel does not scrape audit_log or re-read the bucket.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/model/dona-building-unit-model-draft.xlsx
+++ b/docs/model/dona-building-unit-model-draft.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ENTITIES'!$A$1:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RELATIONSHIPS'!$A$1:$H$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'FIELDS'!$A$1:$G$135</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'FIELDS'!$A$1:$G$136</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ADMIN VIEWS'!$A$1:$E$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DECISIONS'!$A$1:$E$8</definedName>
   </definedNames>
@@ -2010,7 +2010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G135"/>
+  <dimension ref="A1:G136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5137,47 +5137,51 @@
       <c r="F107" s="6" t="inlineStr"/>
       <c r="G107" s="6" t="inlineStr"/>
     </row>
-    <row r="108" ht="20" customHeight="1">
-      <c r="A108" s="7" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>verification_verdict</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr">
+        <is>
+          <t>enum</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E108" s="6" t="inlineStr"/>
+      <c r="F108" s="6" t="inlineStr">
+        <is>
+          <t>verified · unverified · unguarded</t>
+        </is>
+      </c>
+      <c r="G108" s="6" t="inlineStr">
+        <is>
+          <t>Slice 3.6. The 3.3 guard's result, made a property of a list so a scan does not look identical to a lease whose marker terms were found. Not figure 5's state (RECEIVED / EXTRACTED / ACCEPTED / REJECTED), which is still omitted: refused uploads still leave no row. 4.1 may later move unverified → verified once OCR gives the file a text layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="20" customHeight="1">
+      <c r="A109" s="7" t="inlineStr">
         <is>
           <t>E13 · DOCUMENTLINK — one document, several bindings</t>
         </is>
       </c>
-      <c r="B108" s="8" t="n"/>
-      <c r="C108" s="8" t="n"/>
-      <c r="D108" s="8" t="n"/>
-      <c r="E108" s="8" t="n"/>
-      <c r="F108" s="8" t="n"/>
-      <c r="G108" s="8" t="n"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="6" t="inlineStr">
-        <is>
-          <t>DocumentLink</t>
-        </is>
-      </c>
-      <c r="B109" s="6" t="inlineStr">
-        <is>
-          <t>document_id</t>
-        </is>
-      </c>
-      <c r="C109" s="6" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D109" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E109" s="6" t="inlineStr">
-        <is>
-          <t>PK part, FK</t>
-        </is>
-      </c>
-      <c r="F109" s="6" t="inlineStr"/>
-      <c r="G109" s="6" t="inlineStr"/>
+      <c r="B109" s="8" t="n"/>
+      <c r="C109" s="8" t="n"/>
+      <c r="D109" s="8" t="n"/>
+      <c r="E109" s="8" t="n"/>
+      <c r="F109" s="8" t="n"/>
+      <c r="G109" s="8" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
@@ -5187,12 +5191,12 @@
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>entity_type</t>
+          <t>document_id</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D110" s="6" t="inlineStr">
@@ -5200,17 +5204,13 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E110" s="6" t="inlineStr"/>
-      <c r="F110" s="6" t="inlineStr">
-        <is>
-          <t>PROJECT · BUILDING · SPACE · UNIT · TENANCY · PARTY · ASSET · OBLIGATION</t>
-        </is>
-      </c>
-      <c r="G110" s="6" t="inlineStr">
-        <is>
-          <t>PROJECT added by D2 — a tender document belongs to the project, not to any one building.</t>
-        </is>
-      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>PK part, FK</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="inlineStr"/>
+      <c r="G110" s="6" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
@@ -5220,12 +5220,12 @@
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>entity_id</t>
+          <t>entity_type</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
@@ -5233,13 +5233,17 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E111" s="6" t="inlineStr">
-        <is>
-          <t>PK part</t>
-        </is>
-      </c>
-      <c r="F111" s="6" t="inlineStr"/>
-      <c r="G111" s="6" t="inlineStr"/>
+      <c r="E111" s="6" t="inlineStr"/>
+      <c r="F111" s="6" t="inlineStr">
+        <is>
+          <t>PROJECT · BUILDING · SPACE · UNIT · TENANCY · PARTY · ASSET · OBLIGATION</t>
+        </is>
+      </c>
+      <c r="G111" s="6" t="inlineStr">
+        <is>
+          <t>PROJECT added by D2 — a tender document belongs to the project, not to any one building.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
@@ -5249,72 +5253,72 @@
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
+          <t>entity_id</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E112" s="6" t="inlineStr">
+        <is>
+          <t>PK part</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="inlineStr"/>
+      <c r="G112" s="6" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>DocumentLink</t>
+        </is>
+      </c>
+      <c r="B113" s="6" t="inlineStr">
+        <is>
           <t>link_role</t>
         </is>
       </c>
-      <c r="C112" s="6" t="inlineStr">
+      <c r="C113" s="6" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
       </c>
-      <c r="D112" s="6" t="inlineStr">
+      <c r="D113" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="E112" s="6" t="inlineStr"/>
-      <c r="F112" s="6" t="inlineStr">
+      <c r="E113" s="6" t="inlineStr"/>
+      <c r="F113" s="6" t="inlineStr">
         <is>
           <t>SIGNATORY · SUBJECT · EVIDENCE · SOURCE</t>
         </is>
       </c>
-      <c r="G112" s="6" t="inlineStr">
+      <c r="G113" s="6" t="inlineStr">
         <is>
           <t>A lease links to two parties as SIGNATORY and to the unit as SUBJECT.</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="7" t="inlineStr">
+    <row r="114" ht="20" customHeight="1">
+      <c r="A114" s="7" t="inlineStr">
         <is>
           <t>E14 · PROVIDER — stub only, out of scope this pass</t>
         </is>
       </c>
-      <c r="B113" s="8" t="n"/>
-      <c r="C113" s="8" t="n"/>
-      <c r="D113" s="8" t="n"/>
-      <c r="E113" s="8" t="n"/>
-      <c r="F113" s="8" t="n"/>
-      <c r="G113" s="8" t="n"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="6" t="inlineStr">
-        <is>
-          <t>Provider</t>
-        </is>
-      </c>
-      <c r="B114" s="6" t="inlineStr">
-        <is>
-          <t>provider_id</t>
-        </is>
-      </c>
-      <c r="C114" s="6" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D114" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E114" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F114" s="6" t="inlineStr"/>
-      <c r="G114" s="6" t="inlineStr"/>
+      <c r="B114" s="8" t="n"/>
+      <c r="C114" s="8" t="n"/>
+      <c r="D114" s="8" t="n"/>
+      <c r="E114" s="8" t="n"/>
+      <c r="F114" s="8" t="n"/>
+      <c r="G114" s="8" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
@@ -5324,12 +5328,12 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>provider_id</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
@@ -5337,7 +5341,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E115" s="6" t="inlineStr"/>
+      <c r="E115" s="6" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="F115" s="6" t="inlineStr"/>
       <c r="G115" s="6" t="inlineStr"/>
     </row>
@@ -5349,72 +5357,68 @@
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D116" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E116" s="6" t="inlineStr"/>
+      <c r="F116" s="6" t="inlineStr"/>
+      <c r="G116" s="6" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="B117" s="6" t="inlineStr">
+        <is>
           <t>provider_kind</t>
         </is>
       </c>
-      <c r="C116" s="6" t="inlineStr">
+      <c r="C117" s="6" t="inlineStr">
         <is>
           <t>enum</t>
         </is>
       </c>
-      <c r="D116" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E116" s="6" t="inlineStr"/>
-      <c r="F116" s="6" t="inlineStr">
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E117" s="6" t="inlineStr"/>
+      <c r="F117" s="6" t="inlineStr">
         <is>
           <t>IN_HOUSE_CREW · CONTRACTOR · DEVELOPER_WARRANTY</t>
         </is>
       </c>
-      <c r="G116" s="6" t="inlineStr">
+      <c r="G117" s="6" t="inlineStr">
         <is>
           <t>Present only to make R11 resolvable. Everything else about providers waits.</t>
         </is>
       </c>
     </row>
-    <row r="117" ht="20" customHeight="1">
-      <c r="A117" s="7" t="inlineStr">
+    <row r="118" ht="20" customHeight="1">
+      <c r="A118" s="7" t="inlineStr">
         <is>
           <t>E15 · DOCUMENTTYPE — the catalogue behind Document (A8)</t>
         </is>
       </c>
-      <c r="B117" s="8" t="n"/>
-      <c r="C117" s="8" t="n"/>
-      <c r="D117" s="8" t="n"/>
-      <c r="E117" s="8" t="n"/>
-      <c r="F117" s="8" t="n"/>
-      <c r="G117" s="8" t="n"/>
-    </row>
-    <row r="118">
-      <c r="A118" s="6" t="inlineStr">
-        <is>
-          <t>DocumentType</t>
-        </is>
-      </c>
-      <c r="B118" s="6" t="inlineStr">
-        <is>
-          <t>document_type_id</t>
-        </is>
-      </c>
-      <c r="C118" s="6" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D118" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E118" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F118" s="6" t="inlineStr"/>
-      <c r="G118" s="6" t="inlineStr"/>
+      <c r="B118" s="8" t="n"/>
+      <c r="C118" s="8" t="n"/>
+      <c r="D118" s="8" t="n"/>
+      <c r="E118" s="8" t="n"/>
+      <c r="F118" s="8" t="n"/>
+      <c r="G118" s="8" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
@@ -5424,12 +5428,12 @@
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>type_key</t>
+          <t>document_type_id</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
@@ -5439,19 +5443,11 @@
       </c>
       <c r="E119" s="6" t="inlineStr">
         <is>
-          <t>unique</t>
-        </is>
-      </c>
-      <c r="F119" s="6" t="inlineStr">
-        <is>
-          <t>Stable machine key. Nine seed rows: lease · lease_amendment · termination_notice · arnona · insurance · id · bank_guarantee · handover_protocol · inspection_certificate.</t>
-        </is>
-      </c>
-      <c r="G119" s="6" t="inlineStr">
-        <is>
-          <t>The first eight are the Data Model's. inspection_certificate is the ninth, needed by SAFETY assets and by the compliance tab. Never renamed and never reused — filed documents point at it.</t>
-        </is>
-      </c>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="inlineStr"/>
+      <c r="G119" s="6" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="6" t="inlineStr">
@@ -5461,7 +5457,7 @@
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>label_he</t>
+          <t>type_key</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
@@ -5474,13 +5470,21 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E120" s="6" t="inlineStr"/>
+      <c r="E120" s="6" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
       <c r="F120" s="6" t="inlineStr">
         <is>
-          <t>What the admin sees and chooses from: חוזה שכירות · נספח · הודעת סיום · ארנונה · ביטוח · תעודת זהות · ערבות בנקאית · פרוטוקול מסירה · תעודת בדיקה.</t>
-        </is>
-      </c>
-      <c r="G120" s="6" t="inlineStr"/>
+          <t>Stable machine key. Nine seed rows: lease · lease_amendment · termination_notice · arnona · insurance · id · bank_guarantee · handover_protocol · inspection_certificate.</t>
+        </is>
+      </c>
+      <c r="G120" s="6" t="inlineStr">
+        <is>
+          <t>The first eight are the Data Model's. inspection_certificate is the ninth, needed by SAFETY assets and by the compliance tab. Never renamed and never reused — filed documents point at it.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
@@ -5490,7 +5494,7 @@
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>label_en</t>
+          <t>label_he</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
@@ -5500,11 +5504,15 @@
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E121" s="6" t="inlineStr"/>
-      <c r="F121" s="6" t="inlineStr"/>
+      <c r="F121" s="6" t="inlineStr">
+        <is>
+          <t>What the admin sees and chooses from: חוזה שכירות · נספח · הודעת סיום · ארנונה · ביטוח · תעודת זהות · ערבות בנקאית · פרוטוקול מסירה · תעודת בדיקה.</t>
+        </is>
+      </c>
       <c r="G121" s="6" t="inlineStr"/>
     </row>
     <row r="122">
@@ -5515,12 +5523,12 @@
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>verification_terms</t>
+          <t>label_en</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
         <is>
-          <t>text[]</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D122" s="6" t="inlineStr">
@@ -5529,16 +5537,8 @@
         </is>
       </c>
       <c r="E122" s="6" t="inlineStr"/>
-      <c r="F122" s="6" t="inlineStr">
-        <is>
-          <t>Marker terms a document of this type is expected to contain.</t>
-        </is>
-      </c>
-      <c r="G122" s="6" t="inlineStr">
-        <is>
-          <t>The cheap guard in slice 3.3 — right slot, wrong file — reads this and nothing else. It lives on the type row rather than in code, or a new type would arrive with no guard until the next release, and A8 would be true of the catalogue and false of everything that uses it.</t>
-        </is>
-      </c>
+      <c r="F122" s="6" t="inlineStr"/>
+      <c r="G122" s="6" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
@@ -5548,28 +5548,28 @@
       </c>
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>verification_terms</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>text[]</t>
         </is>
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E123" s="6" t="inlineStr"/>
       <c r="F123" s="6" t="inlineStr">
         <is>
-          <t>Retired types stay as rows and stop appearing in the 'file a document' list.</t>
+          <t>Marker terms a document of this type is expected to contain.</t>
         </is>
       </c>
       <c r="G123" s="6" t="inlineStr">
         <is>
-          <t>NEVER delete a type. A9: the admin screen for this catalogue lands in month two; until then we add rows through seeds, which is the same mechanism with a different hand on it.</t>
+          <t>The cheap guard in slice 3.3 — right slot, wrong file — reads this and nothing else. It lives on the type row rather than in code, or a new type would arrive with no guard until the next release, and A8 would be true of the catalogue and false of everything that uses it.</t>
         </is>
       </c>
     </row>
@@ -5581,72 +5581,76 @@
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>is_active</t>
         </is>
       </c>
       <c r="C124" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D124" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E124" s="6" t="inlineStr"/>
       <c r="F124" s="6" t="inlineStr">
         <is>
+          <t>Retired types stay as rows and stop appearing in the 'file a document' list.</t>
+        </is>
+      </c>
+      <c r="G124" s="6" t="inlineStr">
+        <is>
+          <t>NEVER delete a type. A9: the admin screen for this catalogue lands in month two; until then we add rows through seeds, which is the same mechanism with a different hand on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>DocumentType</t>
+        </is>
+      </c>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D125" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E125" s="6" t="inlineStr"/>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
           <t>NO promotes_to. NO validation_rules. NO renewal_cadence.</t>
         </is>
       </c>
-      <c r="G124" s="6" t="inlineStr">
+      <c r="G125" s="6" t="inlineStr">
         <is>
           <t>A8 deliberately: a promotes_to column would make promotion a row, and promotion is the half that is governed — it costs a migration and a reviewed mapping because those columns are what the isolation join, the responsibility matrix and the state machine read. Renewal cadence and 'what is missing' belong to DocumentRequirement, which is month two's.</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="20" customHeight="1">
-      <c r="A125" s="7" t="inlineStr">
+    <row r="126" ht="20" customHeight="1">
+      <c r="A126" s="7" t="inlineStr">
         <is>
           <t>E16 · DOCUMENTTYPEFIELD — what a type declares, in one version (A8)</t>
         </is>
       </c>
-      <c r="B125" s="8" t="n"/>
-      <c r="C125" s="8" t="n"/>
-      <c r="D125" s="8" t="n"/>
-      <c r="E125" s="8" t="n"/>
-      <c r="F125" s="8" t="n"/>
-      <c r="G125" s="8" t="n"/>
-    </row>
-    <row r="126">
-      <c r="A126" s="6" t="inlineStr">
-        <is>
-          <t>DocumentTypeField</t>
-        </is>
-      </c>
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>document_type_field_id</t>
-        </is>
-      </c>
-      <c r="C126" s="6" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="D126" s="6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E126" s="6" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F126" s="6" t="inlineStr"/>
-      <c r="G126" s="6" t="inlineStr"/>
+      <c r="B126" s="8" t="n"/>
+      <c r="C126" s="8" t="n"/>
+      <c r="D126" s="8" t="n"/>
+      <c r="E126" s="8" t="n"/>
+      <c r="F126" s="8" t="n"/>
+      <c r="G126" s="8" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
@@ -5656,7 +5660,7 @@
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>document_type_id</t>
+          <t>document_type_field_id</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
@@ -5671,15 +5675,11 @@
       </c>
       <c r="E127" s="6" t="inlineStr">
         <is>
-          <t>FK → DocumentType</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="F127" s="6" t="inlineStr"/>
-      <c r="G127" s="6" t="inlineStr">
-        <is>
-          <t>See R18.</t>
-        </is>
-      </c>
+      <c r="G127" s="6" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
@@ -5689,12 +5689,12 @@
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>field_key</t>
+          <t>document_type_id</t>
         </is>
       </c>
       <c r="C128" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>id</t>
         </is>
       </c>
       <c r="D128" s="6" t="inlineStr">
@@ -5704,17 +5704,13 @@
       </c>
       <c r="E128" s="6" t="inlineStr">
         <is>
-          <t>unique part</t>
-        </is>
-      </c>
-      <c r="F128" s="6" t="inlineStr">
-        <is>
-          <t>Stable machine key within the type: start_date, end_date, tenant_name, apartment_number.</t>
-        </is>
-      </c>
+          <t>FK → DocumentType</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr"/>
       <c r="G128" s="6" t="inlineStr">
         <is>
-          <t>Unique on (document_type_id, field_key, effective_from) — the same field, redeclared, is a new row and not an edit.</t>
+          <t>See R18.</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5722,7 @@
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>label_he</t>
+          <t>field_key</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
@@ -5739,13 +5735,21 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E129" s="6" t="inlineStr"/>
+      <c r="E129" s="6" t="inlineStr">
+        <is>
+          <t>unique part</t>
+        </is>
+      </c>
       <c r="F129" s="6" t="inlineStr">
         <is>
-          <t>What a reviewer sees beside the value on the page.</t>
-        </is>
-      </c>
-      <c r="G129" s="6" t="inlineStr"/>
+          <t>Stable machine key within the type: start_date, end_date, tenant_name, apartment_number.</t>
+        </is>
+      </c>
+      <c r="G129" s="6" t="inlineStr">
+        <is>
+          <t>Unique on (document_type_id, field_key, effective_from) — the same field, redeclared, is a new row and not an edit.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
@@ -5755,12 +5759,12 @@
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>value_type</t>
+          <t>label_he</t>
         </is>
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D130" s="6" t="inlineStr">
@@ -5771,14 +5775,10 @@
       <c r="E130" s="6" t="inlineStr"/>
       <c r="F130" s="6" t="inlineStr">
         <is>
-          <t>TEXT · NUMBER · DATE · BOOLEAN · ENUM</t>
-        </is>
-      </c>
-      <c r="G130" s="6" t="inlineStr">
-        <is>
-          <t>No MONEY type, and no money field is seeded. READ ME rule 3 binds hardest at promotion: no amount is ever a column on a business record, and no amount is ever quoted to a tenant — the golden set carries that as a standing refusal case.</t>
-        </is>
-      </c>
+          <t>What a reviewer sees beside the value on the page.</t>
+        </is>
+      </c>
+      <c r="G130" s="6" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
@@ -5788,12 +5788,12 @@
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
-          <t>is_required</t>
+          <t>value_type</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="D131" s="6" t="inlineStr">
@@ -5804,12 +5804,12 @@
       <c r="E131" s="6" t="inlineStr"/>
       <c r="F131" s="6" t="inlineStr">
         <is>
-          <t>Is this field expected in a document of this type?</t>
+          <t>TEXT · NUMBER · DATE · BOOLEAN · ENUM</t>
         </is>
       </c>
       <c r="G131" s="6" t="inlineStr">
         <is>
-          <t>A missing required field is a RESULT, not an error. A lease commonly names no guarantor — SPEC-flows A2 — and extraction returning nothing there is correct.</t>
+          <t>No MONEY type, and no money field is seeded. READ ME rule 3 binds hardest at promotion: no amount is ever a column on a business record, and no amount is ever quoted to a tenant — the golden set carries that as a standing refusal case.</t>
         </is>
       </c>
     </row>
@@ -5821,28 +5821,28 @@
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>extraction_hint</t>
+          <t>is_required</t>
         </is>
       </c>
       <c r="C132" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D132" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E132" s="6" t="inlineStr"/>
       <c r="F132" s="6" t="inlineStr">
         <is>
-          <t>The Hebrew phrasing as printed on the form, to look for on the page.</t>
+          <t>Is this field expected in a document of this type?</t>
         </is>
       </c>
       <c r="G132" s="6" t="inlineStr">
         <is>
-          <t>A hint, never a key. Same rule as a Drive path.</t>
+          <t>A missing required field is a RESULT, not an error. A lease commonly names no guarantor — SPEC-flows A2 — and extraction returning nothing there is correct.</t>
         </is>
       </c>
     </row>
@@ -5854,28 +5854,28 @@
       </c>
       <c r="B133" s="6" t="inlineStr">
         <is>
-          <t>effective_from</t>
+          <t>extraction_hint</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E133" s="6" t="inlineStr"/>
       <c r="F133" s="6" t="inlineStr">
         <is>
-          <t>The version. This row governs values extracted on or after this date.</t>
+          <t>The Hebrew phrasing as printed on the form, to look for on the page.</t>
         </is>
       </c>
       <c r="G133" s="6" t="inlineStr">
         <is>
-          <t>A8, for policy_version_id's reason. The extracted value points at THIS row, so A8's schema_version_id is document_type_field_id and there is no separate version entity.</t>
+          <t>A hint, never a key. Same rule as a Drive path.</t>
         </is>
       </c>
     </row>
@@ -5887,7 +5887,7 @@
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>effective_to</t>
+          <t>effective_from</t>
         </is>
       </c>
       <c r="C134" s="6" t="inlineStr">
@@ -5897,18 +5897,18 @@
       </c>
       <c r="D134" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="E134" s="6" t="inlineStr"/>
       <c r="F134" s="6" t="inlineStr">
         <is>
-          <t>Null = the current declaration.</t>
+          <t>The version. This row governs values extracted on or after this date.</t>
         </is>
       </c>
       <c r="G134" s="6" t="inlineStr">
         <is>
-          <t>Closing a row never edits it. Nothing is overwritten — READ ME rule 2.</t>
+          <t>A8, for policy_version_id's reason. The extracted value points at THIS row, so A8's schema_version_id is document_type_field_id and there is no separate version entity.</t>
         </is>
       </c>
     </row>
@@ -5920,33 +5920,66 @@
       </c>
       <c r="B135" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>effective_to</t>
         </is>
       </c>
       <c r="C135" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E135" s="6" t="inlineStr"/>
       <c r="F135" s="6" t="inlineStr">
         <is>
+          <t>Null = the current declaration.</t>
+        </is>
+      </c>
+      <c r="G135" s="6" t="inlineStr">
+        <is>
+          <t>Closing a row never edits it. Nothing is overwritten — READ ME rule 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="6" t="inlineStr">
+        <is>
+          <t>DocumentTypeField</t>
+        </is>
+      </c>
+      <c r="B136" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C136" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D136" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E136" s="6" t="inlineStr"/>
+      <c r="F136" s="6" t="inlineStr">
+        <is>
           <t>NO target column, NO promotion mapping.</t>
         </is>
       </c>
-      <c r="G135" s="6" t="inlineStr">
+      <c r="G136" s="6" t="inlineStr">
         <is>
           <t>Capture is open; promotion is governed. The mapping from a captured field to a typed column is a migration and a reviewed mapping, not a row an admin can add on a Tuesday. See A8.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G135"/>
+  <autoFilter ref="A1:G136"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>